<commit_message>
fixing US universities cost calcualtion error
</commit_message>
<xml_diff>
--- a/fees.xlsx
+++ b/fees.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\Shlok Parekh\Downloads\Course-Verifier-3.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB48CB16-288A-4436-9D56-CD9B184F0152}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{790FA759-3763-498D-AC73-D9A4AF877EC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="601" xr2:uid="{A0B92721-7CDF-495E-B956-6055A365BC29}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2361" uniqueCount="1639">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2364" uniqueCount="1640">
   <si>
     <t>Acharya Nagarjuna University</t>
   </si>
@@ -4968,6 +4968,9 @@
   </si>
   <si>
     <t>Ohio State University</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/10JGWIaOzbsrckLvYq4LKiqHy4_Ri8Rt-/view?usp=sharing</t>
   </si>
 </sst>
 </file>
@@ -14356,8 +14359,16 @@
         <v>1637</v>
       </c>
     </row>
-    <row r="788" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C788" s="22"/>
+    <row r="788" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A788" s="1" t="s">
+        <v>1090</v>
+      </c>
+      <c r="B788" s="1" t="s">
+        <v>1093</v>
+      </c>
+      <c r="C788" s="12" t="s">
+        <v>1639</v>
+      </c>
     </row>
     <row r="789" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C789" s="22"/>
@@ -19773,10 +19784,11 @@
     <hyperlink ref="C598" r:id="rId649" xr:uid="{0A368D49-1F7C-4FA0-82FD-8A76D82CD659}"/>
     <hyperlink ref="C786" r:id="rId650" xr:uid="{B1CFA210-9743-4205-9904-B22C9F9EBED7}"/>
     <hyperlink ref="C787" r:id="rId651" xr:uid="{4D483717-7B75-4C1D-BAF2-3E13CC02FA4B}"/>
+    <hyperlink ref="C788" r:id="rId652" xr:uid="{BA58CA45-509E-4E2D-86A7-BCE34C89B704}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId652"/>
+    <tablePart r:id="rId653"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: switch to nemotron and gemma31b, add madurai keyword
</commit_message>
<xml_diff>
--- a/fees.xlsx
+++ b/fees.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\Shlok Parekh\Downloads\Course-Verifier-3.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C584C692-DEF1-47B8-90F7-239EA9455D49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DB54BE9-9748-4D35-BFEF-A1DDE6F3FAB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="601" xr2:uid="{A0B92721-7CDF-495E-B956-6055A365BC29}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2367" uniqueCount="1642">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2370" uniqueCount="1645">
   <si>
     <t>Acharya Nagarjuna University</t>
   </si>
@@ -4977,6 +4977,15 @@
   </si>
   <si>
     <t>https://drive.google.com/file/d/121extnlXkoHQN1PRdacr7yKqTiQ3P52n/view?usp=sharing</t>
+  </si>
+  <si>
+    <t>Dr. D. Y. Patil Arts, Commerce &amp; Science College, Pimpri, Pune</t>
+  </si>
+  <si>
+    <t>B.Sc (Cyber and Digital Science)</t>
+  </si>
+  <si>
+    <t>https://acs.dypvp.edu.in/DownloadS3File.aspx?file=UG-fee-structure-26-27</t>
   </si>
 </sst>
 </file>
@@ -14384,8 +14393,16 @@
         <v>1638</v>
       </c>
     </row>
-    <row r="790" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C790" s="21"/>
+    <row r="790" spans="1:3" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A790" s="1" t="s">
+        <v>1642</v>
+      </c>
+      <c r="B790" s="1" t="s">
+        <v>1643</v>
+      </c>
+      <c r="C790" s="12" t="s">
+        <v>1644</v>
+      </c>
     </row>
     <row r="791" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C791" s="21"/>
@@ -19799,10 +19816,11 @@
     <hyperlink ref="C328" r:id="rId653" xr:uid="{70C06AF8-BDAF-4E1C-96A2-426717989049}"/>
     <hyperlink ref="C302:C327" r:id="rId654" display="https://drive.google.com/file/d/1rdC7GBkH0w9zhAf2amRYlhGy3XpyonNb/view?usp=sharing" xr:uid="{10D40540-1E43-4456-898C-E35DA9DE0070}"/>
     <hyperlink ref="C329:C331" r:id="rId655" display="https://drive.google.com/file/d/1rdC7GBkH0w9zhAf2amRYlhGy3XpyonNb/view?usp=sharing" xr:uid="{73611974-6B47-494F-B05E-78A491B04B35}"/>
+    <hyperlink ref="C790" r:id="rId656" xr:uid="{5E2299AA-1280-4E52-B85F-61AE3BFCACF0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId656"/>
+    <tablePart r:id="rId657"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>